<commit_message>
#7 Fresh Deliverables generated with client BOM.
</commit_message>
<xml_diff>
--- a/Design-Files/ChargerBoard-v1.1/BOM/Client BOM.xlsx
+++ b/Design-Files/ChargerBoard-v1.1/BOM/Client BOM.xlsx
@@ -5,7 +5,7 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Iftikhar Ahmed\OneDrive\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LiberDB\Documents\GitHub\austingunniers-gamingmouse\Design-Files\ChargerBoard-v1.1\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="237">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="355" uniqueCount="238">
   <si>
     <t>#</t>
   </si>
@@ -75,16 +75,16 @@
     <t>C1</t>
   </si>
   <si>
-    <t>C2</t>
-  </si>
-  <si>
-    <t>C3, C4, C8, C9, C11, C14</t>
+    <t>C2, C28, C29</t>
+  </si>
+  <si>
+    <t>C3, C4, C8, C9, C11, C14, C32</t>
   </si>
   <si>
     <t>C5, C15, C16</t>
   </si>
   <si>
-    <t>C6, C7</t>
+    <t>C6, C7, C31</t>
   </si>
   <si>
     <t>C10</t>
@@ -96,7 +96,7 @@
     <t>C17</t>
   </si>
   <si>
-    <t>C18</t>
+    <t>C18, C30</t>
   </si>
   <si>
     <t>C19</t>
@@ -150,7 +150,7 @@
     <t>LED1</t>
   </si>
   <si>
-    <t>LED2, LED3, LED4, LED5, LED6, LED7, LED8</t>
+    <t>LED3, LED4, LED5, LED6, LED7, LED8</t>
   </si>
   <si>
     <t>R1, R2</t>
@@ -159,19 +159,16 @@
     <t>R3</t>
   </si>
   <si>
-    <t>R4, R5, R7, R8, R9, R12, R13, R18</t>
-  </si>
-  <si>
-    <t>R6</t>
-  </si>
-  <si>
-    <t>R10</t>
-  </si>
-  <si>
-    <t>R11</t>
-  </si>
-  <si>
-    <t>R14, R16, R17</t>
+    <t>R4, R5, R8, R12, R13, R18</t>
+  </si>
+  <si>
+    <t>R6, R10, R11, R14, R16, R17</t>
+  </si>
+  <si>
+    <t>R7</t>
+  </si>
+  <si>
+    <t>R9</t>
   </si>
   <si>
     <t>R15</t>
@@ -201,6 +198,9 @@
     <t>U5</t>
   </si>
   <si>
+    <t>U6</t>
+  </si>
+  <si>
     <t>X1</t>
   </si>
   <si>
@@ -303,21 +303,18 @@
     <t>RES SMD 1M OHM 1% 1/10W 0603</t>
   </si>
   <si>
-    <t>RES 200 OHM 1% 1/16W 0402</t>
-  </si>
-  <si>
-    <t>RES SMD 3.2K OHM 0.1% 1/10W 0603</t>
-  </si>
-  <si>
-    <t>RES SMD 24K OHM 1% 1/16W 0402</t>
-  </si>
-  <si>
-    <t>RES SMD 5.6K OHM 0.1% 1/16W 0402</t>
+    <t>RES 470 OHM 1% 1/16W 0402</t>
   </si>
   <si>
     <t>RES 10K OHM 1% 1/16W 0402</t>
   </si>
   <si>
+    <t>RES 680 OHM 1% 1/16W 0402</t>
+  </si>
+  <si>
+    <t>RES 20K OHM 1% 1/16W 0402</t>
+  </si>
+  <si>
     <t>RES 499 OHM 1% 1/16W 0402</t>
   </si>
   <si>
@@ -330,10 +327,10 @@
     <t>SWITCH TACTILE SPST-NO 0.05A 12V</t>
   </si>
   <si>
-    <t>ESOP-8 Battery Management ICs ROHS</t>
-  </si>
-  <si>
-    <t>DIP-18 Other Lighting Drivers ROHS</t>
+    <t>IC LED DRVR LINEAR 120MA 20TSSOP</t>
+  </si>
+  <si>
+    <t>4.5V~5.5V 锂离子/Polymer 1 600mA SOT-23-5 Battery Management ICs ROHS</t>
   </si>
   <si>
     <t>RF TXRX MODULE BLUETOOTH SMD</t>
@@ -345,6 +342,9 @@
     <t>IC RF TXRX ISM&gt;1GHZ 20VFQFN</t>
   </si>
   <si>
+    <t>IC BATT MON LI-ION 1CELL 8TDFN</t>
+  </si>
+  <si>
     <t>40MHz SMD Crystal Resonator 15pF SMD3225-4P Crystals ROHS</t>
   </si>
   <si>
@@ -393,10 +393,10 @@
     <t>B3U-1000P</t>
   </si>
   <si>
-    <t>ESOP-8</t>
-  </si>
-  <si>
-    <t>DIP-18</t>
+    <t>TSSOP-20</t>
+  </si>
+  <si>
+    <t>SOT-23-5</t>
   </si>
   <si>
     <t>32-QFN (5x5)</t>
@@ -408,6 +408,9 @@
     <t>20-QFN (4x4) EP Via</t>
   </si>
   <si>
+    <t>8-TDFN-EP (2x2)</t>
+  </si>
+  <si>
     <t>SMD3225-4P</t>
   </si>
   <si>
@@ -498,21 +501,18 @@
     <t>RC0603FR-071ML</t>
   </si>
   <si>
-    <t>RC0402FR-07200RL</t>
-  </si>
-  <si>
-    <t>RT0603BRD073K2L</t>
-  </si>
-  <si>
-    <t>RT0402FRE0724KL</t>
-  </si>
-  <si>
-    <t>RT0402BRD075K6L</t>
+    <t>RC0402FR-07470RL</t>
   </si>
   <si>
     <t>RC0402FR-0710KL</t>
   </si>
   <si>
+    <t>RC0402FR-07680RL</t>
+  </si>
+  <si>
+    <t>RC0402FR-0720KL</t>
+  </si>
+  <si>
     <t>RC0402FR-07499RL</t>
   </si>
   <si>
@@ -522,10 +522,10 @@
     <t>AF0402JR-071ML</t>
   </si>
   <si>
-    <t>TP4056-42-ESOP8</t>
-  </si>
-  <si>
-    <t>HT3914ANZ</t>
+    <t>TLC59108FIPWR</t>
+  </si>
+  <si>
+    <t>TP4054</t>
   </si>
   <si>
     <t>ESP32-C3FH4</t>
@@ -537,6 +537,9 @@
     <t>NRF24L01</t>
   </si>
   <si>
+    <t>MAX17048G+T10</t>
+  </si>
+  <si>
     <t>X322540MPB4SI</t>
   </si>
   <si>
@@ -588,10 +591,10 @@
     <t>Omron</t>
   </si>
   <si>
-    <t>TOPPOWER</t>
-  </si>
-  <si>
-    <t>Tae Jin Technology</t>
+    <t>Texas Instruments</t>
+  </si>
+  <si>
+    <t>TPOWER</t>
   </si>
   <si>
     <t>Espressif Systems</t>
@@ -603,6 +606,9 @@
     <t>Nordic Semiconductor</t>
   </si>
   <si>
+    <t>Maxim</t>
+  </si>
+  <si>
     <t>Yangxing Tech</t>
   </si>
   <si>
@@ -678,21 +684,18 @@
     <t>1M</t>
   </si>
   <si>
-    <t>200R</t>
-  </si>
-  <si>
-    <t>3.2K</t>
-  </si>
-  <si>
-    <t>24K</t>
-  </si>
-  <si>
-    <t>5.6K</t>
+    <t>470R</t>
   </si>
   <si>
     <t>10K</t>
   </si>
   <si>
+    <t>680R</t>
+  </si>
+  <si>
+    <t>20K</t>
+  </si>
+  <si>
     <t>499R</t>
   </si>
   <si>
@@ -708,16 +711,16 @@
     <t>Quantity</t>
   </si>
   <si>
+    <t>Remarks</t>
+  </si>
+  <si>
+    <t>Custom</t>
+  </si>
+  <si>
     <t>Value</t>
   </si>
   <si>
-    <t>Remarks</t>
-  </si>
-  <si>
     <t>-</t>
-  </si>
-  <si>
-    <t>Custom</t>
   </si>
   <si>
     <t xml:space="preserve">Peripheral </t>
@@ -941,11 +944,11 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1240,14 +1243,14 @@
   <cols>
     <col min="2" max="2" width="3.140625" style="4" customWidth="1"/>
     <col min="3" max="3" width="18.7109375" style="4" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="36" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="30" customWidth="1"/>
+    <col min="4" max="4" width="27.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="29.85546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="15.7109375" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="33.42578125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="21.42578125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="6.28515625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1259,9 +1262,9 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
-      <c r="I1" s="14"/>
-      <c r="J1" s="14"/>
-      <c r="K1" s="14"/>
+      <c r="I1" s="15"/>
+      <c r="J1" s="15"/>
+      <c r="K1" s="15"/>
     </row>
     <row r="2" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -1281,16 +1284,16 @@
         <v>110</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="I2" s="6" t="s">
+        <v>232</v>
+      </c>
+      <c r="J2" s="5" t="s">
         <v>229</v>
-      </c>
-      <c r="J2" s="5" t="s">
-        <v>228</v>
       </c>
       <c r="K2" s="5" t="s">
         <v>230</v>
@@ -1312,16 +1315,16 @@
         <v>63</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="G3" s="8" t="s">
         <v>111</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="J3" s="7">
         <v>1</v>
@@ -1344,16 +1347,16 @@
         <v>64</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="G4" s="10" t="s">
         <v>112</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="J4" s="9">
         <v>1</v>
@@ -1379,13 +1382,13 @@
         <v>113</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="I5" s="8" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="J5" s="7">
         <v>1</v>
@@ -1411,16 +1414,16 @@
         <v>114</v>
       </c>
       <c r="G6" s="10" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I6" s="10" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="J6" s="9">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K6" s="9"/>
     </row>
@@ -1443,16 +1446,16 @@
         <v>115</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="J7" s="7">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K7" s="7"/>
     </row>
@@ -1475,13 +1478,13 @@
         <v>115</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H8" s="9" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="I8" s="10" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="J8" s="9">
         <v>3</v>
@@ -1507,16 +1510,16 @@
         <v>115</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="I9" s="8" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="J9" s="7">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K9" s="7"/>
     </row>
@@ -1539,13 +1542,13 @@
         <v>115</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="H10" s="9" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="I10" s="10" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="J10" s="9">
         <v>1</v>
@@ -1571,13 +1574,13 @@
         <v>115</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="I11" s="8" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="J11" s="7">
         <v>4</v>
@@ -1603,13 +1606,13 @@
         <v>115</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="H12" s="9" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="I12" s="10" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="J12" s="9">
         <v>1</v>
@@ -1635,16 +1638,16 @@
         <v>115</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="I13" s="8" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="J13" s="7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K13" s="7"/>
     </row>
@@ -1667,13 +1670,13 @@
         <v>115</v>
       </c>
       <c r="G14" s="10" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="H14" s="9" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="J14" s="9">
         <v>1</v>
@@ -1699,13 +1702,13 @@
         <v>115</v>
       </c>
       <c r="G15" s="8" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="I15" s="8" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="J15" s="7">
         <v>1</v>
@@ -1731,13 +1734,13 @@
         <v>115</v>
       </c>
       <c r="G16" s="10" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H16" s="9" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="I16" s="10" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="J16" s="9">
         <v>1</v>
@@ -1763,13 +1766,13 @@
         <v>115</v>
       </c>
       <c r="G17" s="8" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="I17" s="8" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="J17" s="7">
         <v>1</v>
@@ -1795,13 +1798,13 @@
         <v>116</v>
       </c>
       <c r="G18" s="10" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="H18" s="9" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="I18" s="10" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="J18" s="9">
         <v>1</v>
@@ -1827,13 +1830,13 @@
         <v>116</v>
       </c>
       <c r="G19" s="8" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="H19" s="7" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="I19" s="8" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="J19" s="7">
         <v>1</v>
@@ -1859,13 +1862,13 @@
         <v>116</v>
       </c>
       <c r="G20" s="10" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="H20" s="9" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="I20" s="10" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="J20" s="9">
         <v>1</v>
@@ -1888,16 +1891,16 @@
         <v>81</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="G21" s="8" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="H21" s="7" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="I21" s="8" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="J21" s="7">
         <v>1</v>
@@ -1919,17 +1922,17 @@
       <c r="E22" s="10" t="s">
         <v>82</v>
       </c>
-      <c r="F22" s="7" t="s">
-        <v>232</v>
+      <c r="F22" s="9" t="s">
+        <v>231</v>
       </c>
       <c r="G22" s="10" t="s">
         <v>117</v>
       </c>
       <c r="H22" s="9" t="s">
-        <v>182</v>
-      </c>
-      <c r="I22" s="8" t="s">
-        <v>231</v>
+        <v>183</v>
+      </c>
+      <c r="I22" s="10" t="s">
+        <v>233</v>
       </c>
       <c r="J22" s="9">
         <v>1</v>
@@ -1952,16 +1955,16 @@
         <v>83</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="G23" s="8" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="H23" s="7" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="I23" s="8" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="J23" s="7">
         <v>1</v>
@@ -1987,13 +1990,13 @@
         <v>118</v>
       </c>
       <c r="G24" s="10" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="H24" s="9" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="I24" s="10" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="J24" s="9">
         <v>1</v>
@@ -2019,13 +2022,13 @@
         <v>118</v>
       </c>
       <c r="G25" s="8" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="H25" s="7" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="I25" s="8" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="J25" s="7">
         <v>1</v>
@@ -2051,13 +2054,13 @@
         <v>118</v>
       </c>
       <c r="G26" s="10" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="H26" s="9" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="I26" s="10" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="J26" s="9">
         <v>1</v>
@@ -2083,13 +2086,13 @@
         <v>119</v>
       </c>
       <c r="G27" s="8" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="H27" s="7" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="I27" s="8" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="J27" s="7">
         <v>1</v>
@@ -2115,13 +2118,13 @@
         <v>119</v>
       </c>
       <c r="G28" s="10" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="H28" s="9" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="I28" s="10" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="J28" s="9">
         <v>1</v>
@@ -2147,13 +2150,13 @@
         <v>119</v>
       </c>
       <c r="G29" s="8" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="H29" s="7" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="I29" s="8" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="J29" s="7">
         <v>1</v>
@@ -2179,13 +2182,13 @@
         <v>120</v>
       </c>
       <c r="G30" s="10" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="H30" s="9" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="I30" s="10" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="J30" s="9">
         <v>1</v>
@@ -2211,16 +2214,16 @@
         <v>120</v>
       </c>
       <c r="G31" s="8" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="H31" s="7" t="s">
-        <v>186</v>
-      </c>
-      <c r="I31" s="10" t="s">
-        <v>231</v>
+        <v>187</v>
+      </c>
+      <c r="I31" s="8" t="s">
+        <v>233</v>
       </c>
       <c r="J31" s="7">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="K31" s="7"/>
     </row>
@@ -2243,13 +2246,13 @@
         <v>121</v>
       </c>
       <c r="G32" s="10" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="H32" s="9" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="I32" s="10" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="J32" s="9">
         <v>2</v>
@@ -2275,13 +2278,13 @@
         <v>122</v>
       </c>
       <c r="G33" s="8" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="H33" s="7" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="I33" s="8" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="J33" s="7">
         <v>1</v>
@@ -2294,7 +2297,7 @@
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
-      <c r="C34" s="12" t="s">
+      <c r="C34" s="13" t="s">
         <v>10</v>
       </c>
       <c r="D34" s="9" t="s">
@@ -2307,16 +2310,16 @@
         <v>121</v>
       </c>
       <c r="G34" s="10" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="H34" s="9" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="I34" s="10" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="J34" s="9">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="K34" s="9"/>
     </row>
@@ -2336,19 +2339,19 @@
         <v>95</v>
       </c>
       <c r="F35" s="7" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="G35" s="8" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="H35" s="7" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="I35" s="8" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="J35" s="7">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="K35" s="7"/>
     </row>
@@ -2371,13 +2374,13 @@
         <v>121</v>
       </c>
       <c r="G36" s="10" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="H36" s="9" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="I36" s="10" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="J36" s="9">
         <v>1</v>
@@ -2403,13 +2406,13 @@
         <v>121</v>
       </c>
       <c r="G37" s="8" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="H37" s="7" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="I37" s="8" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="J37" s="7">
         <v>1</v>
@@ -2422,7 +2425,7 @@
         <f t="shared" si="0"/>
         <v>36</v>
       </c>
-      <c r="C38" s="13" t="s">
+      <c r="C38" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D38" s="9" t="s">
@@ -2435,16 +2438,16 @@
         <v>121</v>
       </c>
       <c r="G38" s="10" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="H38" s="9" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="I38" s="10" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="J38" s="9">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K38" s="9"/>
     </row>
@@ -2454,7 +2457,7 @@
         <f>ROW(B39) - ROW($B$2)</f>
         <v>37</v>
       </c>
-      <c r="C39" s="13" t="s">
+      <c r="C39" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D39" s="7" t="s">
@@ -2464,16 +2467,16 @@
         <v>99</v>
       </c>
       <c r="F39" s="7" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="G39" s="8" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="H39" s="7" t="s">
-        <v>177</v>
+        <v>188</v>
       </c>
       <c r="I39" s="8" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="J39" s="7">
         <v>1</v>
@@ -2496,16 +2499,16 @@
         <v>100</v>
       </c>
       <c r="F40" s="9" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="G40" s="10" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="H40" s="9" t="s">
-        <v>187</v>
+        <v>178</v>
       </c>
       <c r="I40" s="10" t="s">
-        <v>225</v>
+        <v>220</v>
       </c>
       <c r="J40" s="9">
         <v>1</v>
@@ -2519,7 +2522,7 @@
         <v>39</v>
       </c>
       <c r="C41" s="12" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D41" s="7" t="s">
         <v>53</v>
@@ -2528,19 +2531,19 @@
         <v>101</v>
       </c>
       <c r="F41" s="7" t="s">
-        <v>121</v>
+        <v>231</v>
       </c>
       <c r="G41" s="8" t="s">
-        <v>166</v>
+        <v>123</v>
       </c>
       <c r="H41" s="7" t="s">
-        <v>177</v>
+        <v>189</v>
       </c>
       <c r="I41" s="8" t="s">
-        <v>218</v>
+        <v>233</v>
       </c>
       <c r="J41" s="7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K41" s="7"/>
     </row>
@@ -2551,7 +2554,7 @@
         <v>40</v>
       </c>
       <c r="C42" s="13" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D42" s="9" t="s">
         <v>54</v>
@@ -2560,23 +2563,23 @@
         <v>102</v>
       </c>
       <c r="F42" s="9" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="G42" s="10" t="s">
-        <v>123</v>
+        <v>167</v>
       </c>
       <c r="H42" s="9" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="I42" s="10" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="J42" s="9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K42" s="9"/>
     </row>
-    <row r="43" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" s="1"/>
       <c r="B43" s="11">
         <f>ROW(B43) - ROW($B$2)</f>
@@ -2592,16 +2595,16 @@
         <v>103</v>
       </c>
       <c r="F43" s="7" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="G43" s="8" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="H43" s="7" t="s">
-        <v>189</v>
-      </c>
-      <c r="I43" s="10" t="s">
-        <v>231</v>
+        <v>191</v>
+      </c>
+      <c r="I43" s="8" t="s">
+        <v>233</v>
       </c>
       <c r="J43" s="7">
         <v>1</v>
@@ -2624,16 +2627,16 @@
         <v>104</v>
       </c>
       <c r="F44" s="9" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="G44" s="10" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="H44" s="9" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="I44" s="10" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="J44" s="9">
         <v>1</v>
@@ -2656,16 +2659,16 @@
         <v>105</v>
       </c>
       <c r="F45" s="7" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="G45" s="8" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="H45" s="7" t="s">
-        <v>191</v>
-      </c>
-      <c r="I45" s="10" t="s">
-        <v>231</v>
+        <v>193</v>
+      </c>
+      <c r="I45" s="8" t="s">
+        <v>233</v>
       </c>
       <c r="J45" s="7">
         <v>1</v>
@@ -2688,16 +2691,16 @@
         <v>106</v>
       </c>
       <c r="F46" s="9" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="G46" s="10" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="H46" s="9" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="I46" s="10" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="J46" s="9">
         <v>1</v>
@@ -2720,16 +2723,16 @@
         <v>107</v>
       </c>
       <c r="F47" s="7" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G47" s="8" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="H47" s="7" t="s">
-        <v>193</v>
-      </c>
-      <c r="I47" s="10" t="s">
-        <v>231</v>
+        <v>195</v>
+      </c>
+      <c r="I47" s="8" t="s">
+        <v>233</v>
       </c>
       <c r="J47" s="7">
         <v>1</v>
@@ -2752,16 +2755,16 @@
         <v>108</v>
       </c>
       <c r="F48" s="9" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="G48" s="10" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="H48" s="9" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="I48" s="10" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="J48" s="9">
         <v>1</v>
@@ -2784,16 +2787,16 @@
         <v>109</v>
       </c>
       <c r="F49" s="7" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="G49" s="8" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="H49" s="7" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="I49" s="8" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="J49" s="7">
         <v>1</v>
@@ -2806,62 +2809,64 @@
         <v>48</v>
       </c>
       <c r="C50" s="13" t="s">
+        <v>234</v>
+      </c>
+      <c r="D50" s="9" t="s">
         <v>233</v>
       </c>
-      <c r="D50" s="9" t="s">
-        <v>231</v>
-      </c>
       <c r="E50" s="10" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="F50" s="9" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="G50" s="10" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="H50" s="9" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="I50" s="8" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="J50" s="9">
         <v>1</v>
       </c>
-      <c r="K50" s="9"/>
-    </row>
-    <row r="51" spans="1:11" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K50" s="14" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B51" s="11">
         <f>ROW(B51) - ROW($B$2)</f>
         <v>49</v>
       </c>
       <c r="C51" s="13" t="s">
+        <v>234</v>
+      </c>
+      <c r="D51" s="9" t="s">
         <v>233</v>
       </c>
-      <c r="D51" s="9" t="s">
-        <v>231</v>
-      </c>
       <c r="E51" s="10" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="F51" s="9" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="G51" s="10" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="H51" s="9" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="I51" s="8" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="J51" s="9">
         <v>1</v>
       </c>
-      <c r="K51" s="15" t="s">
-        <v>236</v>
+      <c r="K51" s="14" t="s">
+        <v>237</v>
       </c>
     </row>
   </sheetData>
@@ -2870,8 +2875,9 @@
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="K51" r:id="rId1"/>
+    <hyperlink ref="K50" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
#6 Updated Q1 made BOM File
</commit_message>
<xml_diff>
--- a/Design-Files/ChargerBoard-v1.1/BOM/Client BOM.xlsx
+++ b/Design-Files/ChargerBoard-v1.1/BOM/Client BOM.xlsx
@@ -1,25 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20413"/>
+  <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LiberDB\Documents\GitHub\austingunniers-gamingmouse\Design-Files\ChargerBoard-v1.1\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eSpark\Desktop\BOM file Austin\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18F011C3-2F6E-4D1F-B042-5D53739139B9}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="355" uniqueCount="238">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="376" uniqueCount="254">
   <si>
     <t>#</t>
   </si>
@@ -51,6 +52,9 @@
     <t>LED</t>
   </si>
   <si>
+    <t>Mosfet</t>
+  </si>
+  <si>
     <t>Resistor</t>
   </si>
   <si>
@@ -78,7 +82,7 @@
     <t>C2, C28, C29</t>
   </si>
   <si>
-    <t>C3, C4, C8, C9, C11, C14, C32</t>
+    <t>C3, C4, C8, C9, C11, C14, C32, C33, C34, C35, C36</t>
   </si>
   <si>
     <t>C5, C15, C16</t>
@@ -150,9 +154,15 @@
     <t>LED1</t>
   </si>
   <si>
+    <t>LED2, LED9, LED10, LED11</t>
+  </si>
+  <si>
     <t>LED3, LED4, LED5, LED6, LED7, LED8</t>
   </si>
   <si>
+    <t>Q1</t>
+  </si>
+  <si>
     <t>R1, R2</t>
   </si>
   <si>
@@ -162,7 +172,7 @@
     <t>R4, R5, R8, R12, R13, R18</t>
   </si>
   <si>
-    <t>R6, R10, R11, R14, R16, R17</t>
+    <t>R6, R10, R11, R14, R16, R17, R22</t>
   </si>
   <si>
     <t>R7</t>
@@ -180,6 +190,9 @@
     <t>R20</t>
   </si>
   <si>
+    <t>R23</t>
+  </si>
+  <si>
     <t>SW1, SW2</t>
   </si>
   <si>
@@ -294,9 +307,15 @@
     <t>RED LED 0603 Light Emitting Diodes</t>
   </si>
   <si>
+    <t>SMD,2.4x2.7mm RGB LEDs(Built-in IC) ROHS</t>
+  </si>
+  <si>
     <t>Emerald 0603 Light Emitting Diodes (LED) ROHS</t>
   </si>
   <si>
+    <t>N-CHANNEL 20-V (D-S) MOSFET</t>
+  </si>
+  <si>
     <t>RES 5.1K OHM 1% 1/16W 0402</t>
   </si>
   <si>
@@ -324,6 +343,9 @@
     <t>RES SMD 1M OHM 5% 1/16W 0402</t>
   </si>
   <si>
+    <t>RES SMD 1K OHM 1% 1/5W 0402</t>
+  </si>
+  <si>
     <t>SWITCH TACTILE SPST-NO 0.05A 12V</t>
   </si>
   <si>
@@ -384,6 +406,12 @@
     <t>LED-0603</t>
   </si>
   <si>
+    <t>WS2812C-2427</t>
+  </si>
+  <si>
+    <t>Sot-23</t>
+  </si>
+  <si>
     <t>Res-0402</t>
   </si>
   <si>
@@ -495,6 +523,9 @@
     <t>NCD0603G2</t>
   </si>
   <si>
+    <t>SI2302CDS</t>
+  </si>
+  <si>
     <t>RC0402FR-075K1L</t>
   </si>
   <si>
@@ -522,6 +553,9 @@
     <t>AF0402JR-071ML</t>
   </si>
   <si>
+    <t>CRCW04021K00FKEDHP</t>
+  </si>
+  <si>
     <t>TLC59108FIPWR</t>
   </si>
   <si>
@@ -585,9 +619,18 @@
     <t>Foshan NationStar Optoelectronics</t>
   </si>
   <si>
+    <t>WORLDSEMI</t>
+  </si>
+  <si>
+    <t>TECH PUBLIC</t>
+  </si>
+  <si>
     <t>Vishay</t>
   </si>
   <si>
+    <t>Vishay Dale</t>
+  </si>
+  <si>
     <t>Omron</t>
   </si>
   <si>
@@ -678,6 +721,9 @@
     <t>3.9nH</t>
   </si>
   <si>
+    <t>RED</t>
+  </si>
+  <si>
     <t>5.1K</t>
   </si>
   <si>
@@ -702,6 +748,9 @@
     <t>22K</t>
   </si>
   <si>
+    <t>1K</t>
+  </si>
+  <si>
     <t>40MHz</t>
   </si>
   <si>
@@ -711,34 +760,34 @@
     <t>Quantity</t>
   </si>
   <si>
+    <t xml:space="preserve">Peripheral </t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t xml:space="preserve">USB C-Type Cable </t>
+  </si>
+  <si>
+    <t>Aliexpress</t>
+  </si>
+  <si>
+    <t>Battery</t>
+  </si>
+  <si>
+    <t>Value</t>
+  </si>
+  <si>
     <t>Remarks</t>
   </si>
   <si>
-    <t>Custom</t>
-  </si>
-  <si>
-    <t>Value</t>
-  </si>
-  <si>
-    <t>-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Peripheral </t>
-  </si>
-  <si>
-    <t xml:space="preserve">USB C-Type Cable </t>
-  </si>
-  <si>
-    <t>Battery</t>
-  </si>
-  <si>
-    <t>Aliexpress</t>
+    <t>custom</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1236,20 +1285,20 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:K51"/>
+  <dimension ref="A1:K54"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="4" customWidth="1"/>
     <col min="3" max="3" width="18.7109375" style="4" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="27.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="29.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="36" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="30" customWidth="1"/>
+    <col min="6" max="6" width="26.5703125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="33.42578125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="21.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="6.28515625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="16.7109375" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="10.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1275,28 +1324,28 @@
         <v>1</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>131</v>
+        <v>140</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>175</v>
+        <v>186</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>232</v>
+        <v>251</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>229</v>
+        <v>245</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>230</v>
+        <v>252</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1309,22 +1358,22 @@
         <v>2</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>231</v>
+        <v>253</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>111</v>
+        <v>118</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>176</v>
+        <v>187</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>198</v>
+        <v>212</v>
       </c>
       <c r="J3" s="7">
         <v>1</v>
@@ -1334,29 +1383,29 @@
     <row r="4" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1"/>
       <c r="B4" s="11">
-        <f t="shared" ref="B4:B48" si="0">ROW(B4) - ROW($B$2)</f>
+        <f t="shared" ref="B4:B52" si="0">ROW(B4) - ROW($B$2)</f>
         <v>2</v>
       </c>
       <c r="C4" s="13" t="s">
         <v>2</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>231</v>
+        <v>253</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>112</v>
+        <v>119</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>177</v>
+        <v>188</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>233</v>
+        <v>247</v>
       </c>
       <c r="J4" s="9">
         <v>1</v>
@@ -1373,22 +1422,22 @@
         <v>3</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>113</v>
+        <v>120</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>132</v>
+        <v>141</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>178</v>
+        <v>189</v>
       </c>
       <c r="I5" s="8" t="s">
-        <v>199</v>
+        <v>213</v>
       </c>
       <c r="J5" s="7">
         <v>1</v>
@@ -1401,26 +1450,26 @@
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="C6" s="12" t="s">
+      <c r="C6" s="13" t="s">
         <v>3</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>114</v>
+        <v>121</v>
       </c>
       <c r="G6" s="10" t="s">
-        <v>133</v>
+        <v>142</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>179</v>
+        <v>190</v>
       </c>
       <c r="I6" s="10" t="s">
-        <v>200</v>
+        <v>214</v>
       </c>
       <c r="J6" s="9">
         <v>3</v>
@@ -1433,29 +1482,29 @@
         <f>ROW(B7) - ROW($B$2)</f>
         <v>5</v>
       </c>
-      <c r="C7" s="12" t="s">
+      <c r="C7" s="13" t="s">
         <v>3</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>115</v>
+        <v>122</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>178</v>
+        <v>189</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>201</v>
+        <v>215</v>
       </c>
       <c r="J7" s="7">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="K7" s="7"/>
     </row>
@@ -1469,22 +1518,22 @@
         <v>3</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>115</v>
+        <v>122</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
       <c r="H8" s="9" t="s">
-        <v>178</v>
+        <v>189</v>
       </c>
       <c r="I8" s="10" t="s">
-        <v>202</v>
+        <v>216</v>
       </c>
       <c r="J8" s="9">
         <v>3</v>
@@ -1501,22 +1550,22 @@
         <v>3</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>115</v>
+        <v>122</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>136</v>
+        <v>145</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>178</v>
+        <v>189</v>
       </c>
       <c r="I9" s="8" t="s">
-        <v>203</v>
+        <v>217</v>
       </c>
       <c r="J9" s="7">
         <v>3</v>
@@ -1533,22 +1582,22 @@
         <v>3</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="F10" s="9" t="s">
-        <v>115</v>
+        <v>122</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="H10" s="9" t="s">
-        <v>178</v>
+        <v>189</v>
       </c>
       <c r="I10" s="10" t="s">
-        <v>200</v>
+        <v>214</v>
       </c>
       <c r="J10" s="9">
         <v>1</v>
@@ -1565,22 +1614,22 @@
         <v>3</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>115</v>
+        <v>122</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>138</v>
+        <v>147</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>178</v>
+        <v>189</v>
       </c>
       <c r="I11" s="8" t="s">
-        <v>204</v>
+        <v>218</v>
       </c>
       <c r="J11" s="7">
         <v>4</v>
@@ -1597,22 +1646,22 @@
         <v>3</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="F12" s="9" t="s">
-        <v>115</v>
+        <v>122</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>139</v>
+        <v>148</v>
       </c>
       <c r="H12" s="9" t="s">
-        <v>178</v>
+        <v>189</v>
       </c>
       <c r="I12" s="10" t="s">
-        <v>202</v>
+        <v>216</v>
       </c>
       <c r="J12" s="9">
         <v>1</v>
@@ -1629,22 +1678,22 @@
         <v>3</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>115</v>
+        <v>122</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>140</v>
+        <v>149</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>178</v>
+        <v>189</v>
       </c>
       <c r="I13" s="8" t="s">
-        <v>205</v>
+        <v>219</v>
       </c>
       <c r="J13" s="7">
         <v>2</v>
@@ -1661,22 +1710,22 @@
         <v>3</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="F14" s="9" t="s">
-        <v>115</v>
+        <v>122</v>
       </c>
       <c r="G14" s="10" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="H14" s="9" t="s">
-        <v>178</v>
+        <v>189</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>206</v>
+        <v>220</v>
       </c>
       <c r="J14" s="9">
         <v>1</v>
@@ -1693,22 +1742,22 @@
         <v>3</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>115</v>
+        <v>122</v>
       </c>
       <c r="G15" s="8" t="s">
-        <v>142</v>
+        <v>151</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>180</v>
+        <v>191</v>
       </c>
       <c r="I15" s="8" t="s">
-        <v>207</v>
+        <v>221</v>
       </c>
       <c r="J15" s="7">
         <v>1</v>
@@ -1725,22 +1774,22 @@
         <v>3</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="F16" s="9" t="s">
-        <v>115</v>
+        <v>122</v>
       </c>
       <c r="G16" s="10" t="s">
-        <v>143</v>
+        <v>152</v>
       </c>
       <c r="H16" s="9" t="s">
-        <v>178</v>
+        <v>189</v>
       </c>
       <c r="I16" s="10" t="s">
-        <v>208</v>
+        <v>222</v>
       </c>
       <c r="J16" s="9">
         <v>1</v>
@@ -1757,22 +1806,22 @@
         <v>3</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>115</v>
+        <v>122</v>
       </c>
       <c r="G17" s="8" t="s">
-        <v>144</v>
+        <v>153</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>178</v>
+        <v>189</v>
       </c>
       <c r="I17" s="8" t="s">
-        <v>209</v>
+        <v>223</v>
       </c>
       <c r="J17" s="7">
         <v>1</v>
@@ -1789,22 +1838,22 @@
         <v>3</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="F18" s="9" t="s">
-        <v>116</v>
+        <v>123</v>
       </c>
       <c r="G18" s="10" t="s">
-        <v>145</v>
+        <v>154</v>
       </c>
       <c r="H18" s="9" t="s">
-        <v>181</v>
+        <v>192</v>
       </c>
       <c r="I18" s="10" t="s">
-        <v>210</v>
+        <v>224</v>
       </c>
       <c r="J18" s="9">
         <v>1</v>
@@ -1821,22 +1870,22 @@
         <v>3</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>116</v>
+        <v>123</v>
       </c>
       <c r="G19" s="8" t="s">
-        <v>146</v>
+        <v>155</v>
       </c>
       <c r="H19" s="7" t="s">
-        <v>178</v>
+        <v>189</v>
       </c>
       <c r="I19" s="8" t="s">
-        <v>211</v>
+        <v>225</v>
       </c>
       <c r="J19" s="7">
         <v>1</v>
@@ -1853,22 +1902,22 @@
         <v>3</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="F20" s="9" t="s">
-        <v>116</v>
+        <v>123</v>
       </c>
       <c r="G20" s="10" t="s">
-        <v>147</v>
+        <v>156</v>
       </c>
       <c r="H20" s="9" t="s">
-        <v>178</v>
+        <v>189</v>
       </c>
       <c r="I20" s="10" t="s">
-        <v>212</v>
+        <v>226</v>
       </c>
       <c r="J20" s="9">
         <v>1</v>
@@ -1885,22 +1934,22 @@
         <v>4</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>231</v>
+        <v>253</v>
       </c>
       <c r="G21" s="8" t="s">
-        <v>148</v>
+        <v>157</v>
       </c>
       <c r="H21" s="7" t="s">
-        <v>182</v>
+        <v>193</v>
       </c>
       <c r="I21" s="8" t="s">
-        <v>233</v>
+        <v>247</v>
       </c>
       <c r="J21" s="7">
         <v>1</v>
@@ -1917,22 +1966,22 @@
         <v>5</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E22" s="10" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="F22" s="9" t="s">
-        <v>231</v>
+        <v>253</v>
       </c>
       <c r="G22" s="10" t="s">
-        <v>117</v>
+        <v>124</v>
       </c>
       <c r="H22" s="9" t="s">
-        <v>183</v>
-      </c>
-      <c r="I22" s="10" t="s">
-        <v>233</v>
+        <v>194</v>
+      </c>
+      <c r="I22" s="8" t="s">
+        <v>247</v>
       </c>
       <c r="J22" s="9">
         <v>1</v>
@@ -1949,22 +1998,22 @@
         <v>6</v>
       </c>
       <c r="D23" s="7" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E23" s="8" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>231</v>
+        <v>253</v>
       </c>
       <c r="G23" s="8" t="s">
-        <v>149</v>
+        <v>158</v>
       </c>
       <c r="H23" s="7" t="s">
-        <v>184</v>
+        <v>195</v>
       </c>
       <c r="I23" s="8" t="s">
-        <v>233</v>
+        <v>247</v>
       </c>
       <c r="J23" s="7">
         <v>1</v>
@@ -1981,22 +2030,22 @@
         <v>7</v>
       </c>
       <c r="D24" s="9" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E24" s="10" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="F24" s="9" t="s">
-        <v>118</v>
+        <v>125</v>
       </c>
       <c r="G24" s="10" t="s">
-        <v>150</v>
+        <v>159</v>
       </c>
       <c r="H24" s="9" t="s">
-        <v>185</v>
+        <v>196</v>
       </c>
       <c r="I24" s="10" t="s">
-        <v>213</v>
+        <v>227</v>
       </c>
       <c r="J24" s="9">
         <v>1</v>
@@ -2013,22 +2062,22 @@
         <v>7</v>
       </c>
       <c r="D25" s="7" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E25" s="8" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>118</v>
+        <v>125</v>
       </c>
       <c r="G25" s="8" t="s">
-        <v>151</v>
+        <v>160</v>
       </c>
       <c r="H25" s="7" t="s">
-        <v>177</v>
+        <v>188</v>
       </c>
       <c r="I25" s="8" t="s">
-        <v>214</v>
+        <v>228</v>
       </c>
       <c r="J25" s="7">
         <v>1</v>
@@ -2045,22 +2094,22 @@
         <v>7</v>
       </c>
       <c r="D26" s="9" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E26" s="10" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="F26" s="9" t="s">
-        <v>118</v>
+        <v>125</v>
       </c>
       <c r="G26" s="10" t="s">
-        <v>152</v>
+        <v>161</v>
       </c>
       <c r="H26" s="9" t="s">
-        <v>185</v>
+        <v>196</v>
       </c>
       <c r="I26" s="10" t="s">
-        <v>215</v>
+        <v>229</v>
       </c>
       <c r="J26" s="9">
         <v>1</v>
@@ -2077,22 +2126,22 @@
         <v>8</v>
       </c>
       <c r="D27" s="7" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E27" s="8" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="F27" s="7" t="s">
-        <v>119</v>
+        <v>126</v>
       </c>
       <c r="G27" s="8" t="s">
-        <v>153</v>
+        <v>162</v>
       </c>
       <c r="H27" s="7" t="s">
-        <v>186</v>
+        <v>197</v>
       </c>
       <c r="I27" s="8" t="s">
-        <v>216</v>
+        <v>230</v>
       </c>
       <c r="J27" s="7">
         <v>1</v>
@@ -2109,22 +2158,22 @@
         <v>7</v>
       </c>
       <c r="D28" s="9" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E28" s="10" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="F28" s="9" t="s">
-        <v>119</v>
+        <v>126</v>
       </c>
       <c r="G28" s="10" t="s">
-        <v>154</v>
+        <v>163</v>
       </c>
       <c r="H28" s="9" t="s">
-        <v>185</v>
+        <v>196</v>
       </c>
       <c r="I28" s="10" t="s">
-        <v>217</v>
+        <v>231</v>
       </c>
       <c r="J28" s="9">
         <v>1</v>
@@ -2141,22 +2190,22 @@
         <v>7</v>
       </c>
       <c r="D29" s="7" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E29" s="8" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="F29" s="7" t="s">
-        <v>119</v>
+        <v>126</v>
       </c>
       <c r="G29" s="8" t="s">
-        <v>155</v>
+        <v>164</v>
       </c>
       <c r="H29" s="7" t="s">
-        <v>186</v>
+        <v>197</v>
       </c>
       <c r="I29" s="8" t="s">
-        <v>218</v>
+        <v>232</v>
       </c>
       <c r="J29" s="7">
         <v>1</v>
@@ -2173,19 +2222,19 @@
         <v>9</v>
       </c>
       <c r="D30" s="9" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E30" s="10" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="F30" s="9" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="G30" s="10" t="s">
-        <v>156</v>
+        <v>165</v>
       </c>
       <c r="H30" s="9" t="s">
-        <v>187</v>
+        <v>198</v>
       </c>
       <c r="I30" s="10" t="s">
         <v>233</v>
@@ -2205,57 +2254,57 @@
         <v>9</v>
       </c>
       <c r="D31" s="7" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E31" s="8" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="F31" s="7" t="s">
-        <v>120</v>
+        <v>253</v>
       </c>
       <c r="G31" s="8" t="s">
-        <v>157</v>
+        <v>128</v>
       </c>
       <c r="H31" s="7" t="s">
-        <v>187</v>
+        <v>199</v>
       </c>
       <c r="I31" s="8" t="s">
-        <v>233</v>
+        <v>247</v>
       </c>
       <c r="J31" s="7">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="K31" s="7"/>
     </row>
-    <row r="32" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="1"/>
       <c r="B32" s="11">
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
       <c r="C32" s="13" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D32" s="9" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E32" s="10" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="F32" s="9" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="G32" s="10" t="s">
-        <v>158</v>
+        <v>166</v>
       </c>
       <c r="H32" s="9" t="s">
-        <v>178</v>
+        <v>198</v>
       </c>
       <c r="I32" s="10" t="s">
-        <v>219</v>
+        <v>247</v>
       </c>
       <c r="J32" s="9">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="K32" s="9"/>
     </row>
@@ -2269,22 +2318,22 @@
         <v>10</v>
       </c>
       <c r="D33" s="7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E33" s="8" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="F33" s="7" t="s">
-        <v>122</v>
+        <v>129</v>
       </c>
       <c r="G33" s="8" t="s">
-        <v>159</v>
+        <v>167</v>
       </c>
       <c r="H33" s="7" t="s">
-        <v>178</v>
+        <v>200</v>
       </c>
       <c r="I33" s="8" t="s">
-        <v>220</v>
+        <v>247</v>
       </c>
       <c r="J33" s="7">
         <v>1</v>
@@ -2298,28 +2347,28 @@
         <v>32</v>
       </c>
       <c r="C34" s="13" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D34" s="9" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E34" s="10" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="F34" s="9" t="s">
-        <v>121</v>
+        <v>130</v>
       </c>
       <c r="G34" s="10" t="s">
-        <v>160</v>
+        <v>168</v>
       </c>
       <c r="H34" s="9" t="s">
-        <v>178</v>
+        <v>189</v>
       </c>
       <c r="I34" s="10" t="s">
-        <v>221</v>
+        <v>234</v>
       </c>
       <c r="J34" s="9">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="K34" s="9"/>
     </row>
@@ -2330,28 +2379,28 @@
         <v>33</v>
       </c>
       <c r="C35" s="12" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D35" s="7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E35" s="8" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="F35" s="7" t="s">
-        <v>121</v>
+        <v>131</v>
       </c>
       <c r="G35" s="8" t="s">
-        <v>161</v>
+        <v>169</v>
       </c>
       <c r="H35" s="7" t="s">
-        <v>178</v>
+        <v>189</v>
       </c>
       <c r="I35" s="8" t="s">
-        <v>222</v>
+        <v>235</v>
       </c>
       <c r="J35" s="7">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="K35" s="7"/>
     </row>
@@ -2362,28 +2411,28 @@
         <v>34</v>
       </c>
       <c r="C36" s="13" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D36" s="9" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E36" s="10" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="F36" s="9" t="s">
-        <v>121</v>
+        <v>130</v>
       </c>
       <c r="G36" s="10" t="s">
-        <v>162</v>
+        <v>170</v>
       </c>
       <c r="H36" s="9" t="s">
-        <v>178</v>
+        <v>189</v>
       </c>
       <c r="I36" s="10" t="s">
-        <v>223</v>
+        <v>236</v>
       </c>
       <c r="J36" s="9">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="K36" s="9"/>
     </row>
@@ -2394,28 +2443,28 @@
         <v>35</v>
       </c>
       <c r="C37" s="12" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D37" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E37" s="8" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="F37" s="7" t="s">
-        <v>121</v>
+        <v>130</v>
       </c>
       <c r="G37" s="8" t="s">
-        <v>163</v>
+        <v>171</v>
       </c>
       <c r="H37" s="7" t="s">
-        <v>178</v>
+        <v>189</v>
       </c>
       <c r="I37" s="8" t="s">
-        <v>224</v>
+        <v>237</v>
       </c>
       <c r="J37" s="7">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="K37" s="7"/>
     </row>
@@ -2425,26 +2474,26 @@
         <f t="shared" si="0"/>
         <v>36</v>
       </c>
-      <c r="C38" s="12" t="s">
-        <v>10</v>
+      <c r="C38" s="13" t="s">
+        <v>11</v>
       </c>
       <c r="D38" s="9" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E38" s="10" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="F38" s="9" t="s">
-        <v>121</v>
+        <v>130</v>
       </c>
       <c r="G38" s="10" t="s">
-        <v>164</v>
+        <v>172</v>
       </c>
       <c r="H38" s="9" t="s">
-        <v>178</v>
+        <v>189</v>
       </c>
       <c r="I38" s="10" t="s">
-        <v>225</v>
+        <v>238</v>
       </c>
       <c r="J38" s="9">
         <v>1</v>
@@ -2458,25 +2507,25 @@
         <v>37</v>
       </c>
       <c r="C39" s="12" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D39" s="7" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E39" s="8" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="F39" s="7" t="s">
-        <v>122</v>
+        <v>130</v>
       </c>
       <c r="G39" s="8" t="s">
-        <v>165</v>
+        <v>173</v>
       </c>
       <c r="H39" s="7" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="I39" s="8" t="s">
-        <v>226</v>
+        <v>239</v>
       </c>
       <c r="J39" s="7">
         <v>1</v>
@@ -2489,26 +2538,26 @@
         <f t="shared" si="0"/>
         <v>38</v>
       </c>
-      <c r="C40" s="13" t="s">
-        <v>10</v>
+      <c r="C40" s="12" t="s">
+        <v>11</v>
       </c>
       <c r="D40" s="9" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E40" s="10" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="F40" s="9" t="s">
-        <v>121</v>
+        <v>130</v>
       </c>
       <c r="G40" s="10" t="s">
-        <v>166</v>
+        <v>174</v>
       </c>
       <c r="H40" s="9" t="s">
-        <v>178</v>
+        <v>189</v>
       </c>
       <c r="I40" s="10" t="s">
-        <v>220</v>
+        <v>240</v>
       </c>
       <c r="J40" s="9">
         <v>1</v>
@@ -2525,25 +2574,25 @@
         <v>11</v>
       </c>
       <c r="D41" s="7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E41" s="8" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="F41" s="7" t="s">
-        <v>231</v>
+        <v>131</v>
       </c>
       <c r="G41" s="8" t="s">
-        <v>123</v>
+        <v>175</v>
       </c>
       <c r="H41" s="7" t="s">
-        <v>189</v>
+        <v>201</v>
       </c>
       <c r="I41" s="8" t="s">
-        <v>233</v>
+        <v>241</v>
       </c>
       <c r="J41" s="7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K41" s="7"/>
     </row>
@@ -2554,57 +2603,57 @@
         <v>40</v>
       </c>
       <c r="C42" s="13" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D42" s="9" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E42" s="10" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="F42" s="9" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="G42" s="10" t="s">
-        <v>167</v>
+        <v>176</v>
       </c>
       <c r="H42" s="9" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="I42" s="10" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="J42" s="9">
         <v>1</v>
       </c>
       <c r="K42" s="9"/>
     </row>
-    <row r="43" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" s="1"/>
       <c r="B43" s="11">
         <f>ROW(B43) - ROW($B$2)</f>
         <v>41</v>
       </c>
-      <c r="C43" s="12" t="s">
-        <v>12</v>
+      <c r="C43" s="13" t="s">
+        <v>11</v>
       </c>
       <c r="D43" s="7" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E43" s="8" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="F43" s="7" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="G43" s="8" t="s">
-        <v>168</v>
+        <v>177</v>
       </c>
       <c r="H43" s="7" t="s">
-        <v>191</v>
+        <v>202</v>
       </c>
       <c r="I43" s="8" t="s">
-        <v>233</v>
+        <v>242</v>
       </c>
       <c r="J43" s="7">
         <v>1</v>
@@ -2621,25 +2670,25 @@
         <v>12</v>
       </c>
       <c r="D44" s="9" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E44" s="10" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="F44" s="9" t="s">
-        <v>126</v>
+        <v>253</v>
       </c>
       <c r="G44" s="10" t="s">
-        <v>169</v>
+        <v>132</v>
       </c>
       <c r="H44" s="9" t="s">
-        <v>192</v>
+        <v>203</v>
       </c>
       <c r="I44" s="10" t="s">
-        <v>233</v>
+        <v>247</v>
       </c>
       <c r="J44" s="9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K44" s="9"/>
     </row>
@@ -2650,57 +2699,57 @@
         <v>43</v>
       </c>
       <c r="C45" s="12" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D45" s="7" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E45" s="8" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="F45" s="7" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="G45" s="8" t="s">
-        <v>170</v>
+        <v>178</v>
       </c>
       <c r="H45" s="7" t="s">
-        <v>193</v>
+        <v>204</v>
       </c>
       <c r="I45" s="8" t="s">
-        <v>233</v>
+        <v>247</v>
       </c>
       <c r="J45" s="7">
         <v>1</v>
       </c>
       <c r="K45" s="7"/>
     </row>
-    <row r="46" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A46" s="1"/>
       <c r="B46" s="11">
         <f t="shared" si="0"/>
         <v>44</v>
       </c>
       <c r="C46" s="13" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D46" s="9" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E46" s="10" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="F46" s="9" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="G46" s="10" t="s">
-        <v>171</v>
+        <v>179</v>
       </c>
       <c r="H46" s="9" t="s">
-        <v>194</v>
+        <v>205</v>
       </c>
       <c r="I46" s="10" t="s">
-        <v>233</v>
+        <v>247</v>
       </c>
       <c r="J46" s="9">
         <v>1</v>
@@ -2714,32 +2763,32 @@
         <v>45</v>
       </c>
       <c r="C47" s="12" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D47" s="7" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E47" s="8" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="F47" s="7" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="G47" s="8" t="s">
-        <v>172</v>
+        <v>180</v>
       </c>
       <c r="H47" s="7" t="s">
-        <v>195</v>
-      </c>
-      <c r="I47" s="8" t="s">
-        <v>233</v>
+        <v>206</v>
+      </c>
+      <c r="I47" s="10" t="s">
+        <v>247</v>
       </c>
       <c r="J47" s="7">
         <v>1</v>
       </c>
       <c r="K47" s="7"/>
     </row>
-    <row r="48" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A48" s="1"/>
       <c r="B48" s="11">
         <f t="shared" si="0"/>
@@ -2749,29 +2798,29 @@
         <v>13</v>
       </c>
       <c r="D48" s="9" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E48" s="10" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="F48" s="9" t="s">
-        <v>231</v>
+        <v>136</v>
       </c>
       <c r="G48" s="10" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="H48" s="9" t="s">
-        <v>196</v>
+        <v>207</v>
       </c>
       <c r="I48" s="10" t="s">
-        <v>227</v>
+        <v>247</v>
       </c>
       <c r="J48" s="9">
         <v>1</v>
       </c>
       <c r="K48" s="9"/>
     </row>
-    <row r="49" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A49" s="1"/>
       <c r="B49" s="11">
         <f>ROW(B49) - ROW($B$2)</f>
@@ -2781,22 +2830,22 @@
         <v>13</v>
       </c>
       <c r="D49" s="7" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="E49" s="8" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="F49" s="7" t="s">
-        <v>130</v>
+        <v>137</v>
       </c>
       <c r="G49" s="8" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="H49" s="7" t="s">
-        <v>197</v>
-      </c>
-      <c r="I49" s="8" t="s">
-        <v>228</v>
+        <v>208</v>
+      </c>
+      <c r="I49" s="10" t="s">
+        <v>247</v>
       </c>
       <c r="J49" s="7">
         <v>1</v>
@@ -2804,69 +2853,165 @@
       <c r="K49" s="7"/>
     </row>
     <row r="50" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A50" s="1"/>
       <c r="B50" s="11">
-        <f>ROW(B50) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>48</v>
       </c>
       <c r="C50" s="13" t="s">
-        <v>234</v>
+        <v>13</v>
       </c>
       <c r="D50" s="9" t="s">
-        <v>233</v>
+        <v>63</v>
       </c>
       <c r="E50" s="10" t="s">
-        <v>233</v>
+        <v>114</v>
       </c>
       <c r="F50" s="9" t="s">
-        <v>233</v>
+        <v>138</v>
       </c>
       <c r="G50" s="10" t="s">
-        <v>235</v>
+        <v>183</v>
       </c>
       <c r="H50" s="9" t="s">
-        <v>233</v>
-      </c>
-      <c r="I50" s="8" t="s">
-        <v>233</v>
+        <v>209</v>
+      </c>
+      <c r="I50" s="10" t="s">
+        <v>247</v>
       </c>
       <c r="J50" s="9">
         <v>1</v>
       </c>
-      <c r="K50" s="14" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="51" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K50" s="9"/>
+    </row>
+    <row r="51" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A51" s="1"/>
       <c r="B51" s="11">
         <f>ROW(B51) - ROW($B$2)</f>
         <v>49</v>
       </c>
-      <c r="C51" s="13" t="s">
-        <v>234</v>
-      </c>
-      <c r="D51" s="9" t="s">
-        <v>233</v>
-      </c>
-      <c r="E51" s="10" t="s">
-        <v>233</v>
-      </c>
-      <c r="F51" s="9" t="s">
-        <v>233</v>
-      </c>
-      <c r="G51" s="10" t="s">
-        <v>236</v>
-      </c>
-      <c r="H51" s="9" t="s">
-        <v>233</v>
+      <c r="C51" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D51" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="E51" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="F51" s="7" t="s">
+        <v>253</v>
+      </c>
+      <c r="G51" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="H51" s="7" t="s">
+        <v>210</v>
       </c>
       <c r="I51" s="8" t="s">
-        <v>233</v>
-      </c>
-      <c r="J51" s="9">
-        <v>1</v>
-      </c>
-      <c r="K51" s="14" t="s">
-        <v>237</v>
+        <v>243</v>
+      </c>
+      <c r="J51" s="7">
+        <v>1</v>
+      </c>
+      <c r="K51" s="7"/>
+    </row>
+    <row r="52" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A52" s="1"/>
+      <c r="B52" s="11">
+        <f t="shared" si="0"/>
+        <v>50</v>
+      </c>
+      <c r="C52" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="D52" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="E52" s="10" t="s">
+        <v>116</v>
+      </c>
+      <c r="F52" s="9" t="s">
+        <v>139</v>
+      </c>
+      <c r="G52" s="10" t="s">
+        <v>185</v>
+      </c>
+      <c r="H52" s="9" t="s">
+        <v>211</v>
+      </c>
+      <c r="I52" s="10" t="s">
+        <v>244</v>
+      </c>
+      <c r="J52" s="9">
+        <v>1</v>
+      </c>
+      <c r="K52" s="9"/>
+    </row>
+    <row r="53" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B53" s="11">
+        <f>ROW(B53) - ROW($B$2)</f>
+        <v>51</v>
+      </c>
+      <c r="C53" s="13" t="s">
+        <v>246</v>
+      </c>
+      <c r="D53" s="9" t="s">
+        <v>247</v>
+      </c>
+      <c r="E53" s="10" t="s">
+        <v>247</v>
+      </c>
+      <c r="F53" s="9" t="s">
+        <v>247</v>
+      </c>
+      <c r="G53" s="10" t="s">
+        <v>248</v>
+      </c>
+      <c r="H53" s="9" t="s">
+        <v>247</v>
+      </c>
+      <c r="I53" s="8" t="s">
+        <v>247</v>
+      </c>
+      <c r="J53" s="9">
+        <v>1</v>
+      </c>
+      <c r="K53" s="14" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="54" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B54" s="11">
+        <f>ROW(B54) - ROW($B$2)</f>
+        <v>52</v>
+      </c>
+      <c r="C54" s="13" t="s">
+        <v>246</v>
+      </c>
+      <c r="D54" s="9" t="s">
+        <v>247</v>
+      </c>
+      <c r="E54" s="10" t="s">
+        <v>247</v>
+      </c>
+      <c r="F54" s="9" t="s">
+        <v>247</v>
+      </c>
+      <c r="G54" s="10" t="s">
+        <v>250</v>
+      </c>
+      <c r="H54" s="9" t="s">
+        <v>247</v>
+      </c>
+      <c r="I54" s="8" t="s">
+        <v>247</v>
+      </c>
+      <c r="J54" s="9">
+        <v>1</v>
+      </c>
+      <c r="K54" s="14" t="s">
+        <v>249</v>
       </c>
     </row>
   </sheetData>
@@ -2874,8 +3019,8 @@
     <mergeCell ref="I1:K1"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="K51" r:id="rId1"/>
-    <hyperlink ref="K50" r:id="rId2"/>
+    <hyperlink ref="K54" r:id="rId1" xr:uid="{932F8D24-B32A-4B53-89BA-BFC2A6C82531}"/>
+    <hyperlink ref="K53" r:id="rId2" xr:uid="{347E8977-D0FA-4143-A92B-E15B926D98C0}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId3"/>

</xml_diff>